<commit_message>
N1 语料轨判定: LP AUPRC 0.6870 vs B0 0.7177 (Δ-3.07pt) 不过线,G2 取消,主线维持 PTB-XL 单库;台账/RunLog 归档
</commit_message>
<xml_diff>
--- a/LFBT实验方向清单.xlsx
+++ b/LFBT实验方向清单.xlsx
@@ -1492,7 +1492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1665,6 +1665,28 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="70" customHeight="1">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>#N1判定</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>N1 多库语料轨判死:LP AUPRC 0.6870 vs B0 0.7177(Δ−3.07pt),不满足'PTB-XL≥B0'主判据;主线维持 PTB-XL 单库语料</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>异质语料稀释 PTB-XL 特异形态;混合比例/两阶段课程为附录级改道,不占主线;省 GPU(粗筛 1.4h/次)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B2:E2"/>

</xml_diff>